<commit_message>
geracao de volumes com bases em producao
</commit_message>
<xml_diff>
--- a/bancos/manual/desc_fontes_de_recursos_stn.xlsx
+++ b/bancos/manual/desc_fontes_de_recursos_stn.xlsx
@@ -351,7 +351,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C88"/>
+  <dimension ref="A1:C94"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" s="1" customFormat="1">
@@ -377,7 +377,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Recursos não Vinculados de Impostos</t>
+          <t>RECURSOS NÃO VINCULADOS DE IMPOSTOS</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -392,7 +392,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Outros Recursos não Vinculados</t>
+          <t>OUTROS RECURSOS NÃO VINCULADOS</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -407,7 +407,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Recursos não vinculados da compensação de impostos.</t>
+          <t>RECURSOS NÃO VINCULADOS DA COMPENSAÇÃO DE IMPOSTOS.</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -418,1259 +418,1349 @@
     </row>
     <row r="5">
       <c r="A5">
-        <v>540</v>
+        <v>503</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Transferências do FUNDEB - Impostos e Transferências de Impostos</t>
+          <t>APOIO FINANCEIRO DA UNIÃO EM DECORRÊNCIA DE ESTADO DE CALAMIDADE PÚBLICA.</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Controle dos recursos recebidos do FUNDEB referente à repartição dentro de cada Estado, com base nos incisos I, II e III do art. 212-A da Constituição Federal. Na fase da despesa, quando for o caso, será necessário associar esta fonte ao marcador do percentual de aplicação no pagamento da remuneração dos profissionais da educação básica em efetivo exercício para identificar o cumprimento do percentual mínimo de 70% estabelecido no inciso XI do art. 212-A da CF.</t>
+          <t>Controle dos recursos transferidos pela União a título de apoio financeiro com o objetivo  de enfrentar situações de calamidade pública e suas consequências sociais e econômicas, como  o apoio financeiro decorrente da Medida Provisória n° 1.222, de 21 de maio de 2024.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Transferências do FUNDEB - Complementação da União - VAAF</t>
+          <t>TRANSFERÊNCIAS DO FUNDEB - IMPOSTOS E TRANSFERÊNCIAS DE IMPOSTOS</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Controle dos recursos de complementação da União ao FUNDEB - VAAF, com base na alínea a do inciso V do art. 212-A da Constituição Federal. Na fase da despesa, quando for o caso, será necessário associar esta fonte ao marcador do percentual de aplicação no pagamento da remuneração dos profissionais da educação básica em efetivo exercício para identificar o cumprimento do percentual mínimo de 70% estabelecido no inciso XI do art. 212-A da CF.</t>
+          <t>Controle dos recursos recebidos do FUNDEB referente à repartição dentro de cada Estado, com base nos incisos I, II e III do art. 212-A da Constituição Federal. Na fase da despesa, quando for o caso, será necessário associar esta fonte ao marcador do percentual de aplicação no pagamento da remuneração dos profissionais da educação básica em efetivo exercício para identificar o cumprimento do percentual mínimo de 70% estabelecido no inciso XI do art. 212-A da CF.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Transferências do FUNDEB - Complementação da União - VAAT</t>
+          <t>TRANSFERÊNCIAS DO FUNDEB - COMPLEMENTAÇÃO DA UNIÃO - VAAF</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Controle dos recursos de complementação da União ao FUNDEB - VAAT, com base na alínea b do inciso V do art. 212-A da Constituição Federal. Na fase da despesa, quando for o caso, será necessário associar esta fonte ao marcador do percentual de aplicação no pagamento da remuneração dos profissionais da educação básica em efetivo exercício para identificar o cumprimento do percentual mínimo de 70% estabelecido no inciso XI do art. 212-A da CF.</t>
+          <t>Controle dos recursos de complementação da União ao FUNDEB - VAAF, com base na alínea a do inciso V do art. 212-A da Constituição Federal. Na fase da despesa, quando for o caso, será necessário associar esta fonte ao marcador do percentual de aplicação no pagamento da remuneração dos profissionais da educação básica em efetivo exercício para identificar o cumprimento do percentual mínimo de 70% estabelecido no inciso XI do art. 212-A da CF.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Transferências do FUNDEB - Complementação da União - VAAR</t>
+          <t>TRANSFERÊNCIAS DO FUNDEB - COMPLEMENTAÇÃO DA UNIÃO - VAAT</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Controle dos recursos de complementação da União ao FUNDEB - VAAR, com base na alínea c, inciso V do art. 212-A da Constituição Federal.</t>
+          <t>Controle dos recursos de complementação da União ao FUNDEB - VAAT, com base na alínea b do inciso V do art. 212-A da Constituição Federal. Na fase da despesa, quando for o caso, será necessário associar esta fonte ao marcador do percentual de aplicação no pagamento da remuneração dos profissionais da educação básica em efetivo exercício para identificar o cumprimento do percentual mínimo de 70% estabelecido no inciso XI do art. 212-A da CF.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Recursos de Precatórios do FUNDEF</t>
+          <t>TRANSFERÊNCIAS DO FUNDEB - COMPLEMENTAÇÃO DA UNIÃO - VAAR</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Controle dos recursos decorrentes do recebimento de precatórios derivados de ações judiciais associadas à complementação devida pela União ao Fundo de Manutenção e Desenvolvimento do Ensino Fundamental e de Valorização do Magistério dos demais entes federados (Precatórios Fundef).</t>
+          <t>Controle dos recursos de complementação da União ao FUNDEB - VAAR, com base na alínea c, inciso V do art. 212-A da Constituição Federal.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>550</v>
+        <v>544</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Transferência do Salário-Educação</t>
+          <t>RECURSOS DE PRECATÓRIOS DO FUNDEF</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências recebidas do Fundo Nacional do Desenvolvimento da Educação - FNDE, relativos aos repasses referentes ao salário-educação.</t>
+          <t>Controle dos recursos decorrentes do recebimento de precatórios derivados de ações judiciais associadas à complementação devida pela União ao Fundo de Manutenção e Desenvolvimento do Ensino Fundamental e de Valorização do Magistério dos demais entes federados (Precatórios Fundef).</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11">
-        <v>551</v>
+        <v>545</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Transferências de Recursos do FNDE referentes ao Programa Dinheiro Direto na Escola (PDDE)</t>
+          <t>RECURSOS DE PRECATÓRIOS DO FUNDEB (2007- 2020)</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências do Fundo Nacional do Desenvolvimento da Educação - FNDE, destinados ao Programa Dinheiro Direto na Escola (PDDE).</t>
+          <t>Controle dos recursos decorrentes do recebimento de precatórios derivados de ações  judiciais associadas aos repasses ao Fundo de Manutenção e Desenvolvimento da Educação  Básica e de Valorização dos Profissionais da Educação (Fundeb) 2007-2020, para atendimento  ao previsto no artigo 47-A da Lei nº 14.113, de 25 de dezembro de 2020.</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>552</v>
+        <v>550</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Transferências de Recursos do FNDE referentes ao Programa Nacional de Alimentação Escolar (PNAE)</t>
+          <t>TRANSFERÊNCIA DO SALÁRIO-EDUCAÇÃO</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências do Fundo Nacional do Desenvolvimento da Educação - FNDE, destinados ao Programa Nacional de Alimentação Escolar (PNAE).</t>
+          <t>Controle dos recursos originários de transferências recebidas do Fundo Nacional do Desenvolvimento da Educação - FNDE, relativos aos repasses referentes ao salário-educação.</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>553</v>
+        <v>551</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Transferências de Recursos do FNDE Referentes ao Programa Nacional de Apoio ao Transporte Escolar (PNATE)</t>
+          <t>TRANSFERÊNCIAS DE RECURSOS DO FNDE REFERENTES AO PROGRAMA DINHEIRO DIRETO NA ESCOLA (PDDE)</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências do Fundo Nacional do Desenvolvimento da Educação - FNDE, destinados ao Programa Nacional de Apoio ao Transporte Escolar (PNATE).</t>
+          <t>Controle dos recursos originários de transferências do Fundo Nacional do Desenvolvimento da Educação - FNDE, destinados ao Programa Dinheiro Direto na Escola (PDDE).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14">
-        <v>569</v>
+        <v>552</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Outras Transferências de Recursos do FNDE</t>
+          <t>TRANSFERÊNCIAS DE RECURSOS DO FNDE REFERENTES AO PROGRAMA NACIONAL DE ALIMENTAÇÃO ESCOLAR (PNAE)</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Controle dos demais recursos originários de transferências do Fundo Nacional do Desenvolvimento da Educação - FNDE.</t>
+          <t>Controle dos recursos originários de transferências do Fundo Nacional do Desenvolvimento da Educação - FNDE, destinados ao Programa Nacional de Alimentação Escolar (PNAE).</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15">
-        <v>570</v>
+        <v>553</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Transferências do Governo Federal referentes a Convênios e Instrumentos Congêneres vinculados à Educação</t>
+          <t>TRANSFERÊNCIAS DE RECURSOS DO FNDE REFERENTES AO PROGRAMA NACIONAL DE APOIO AO TRANSPORTE ESCOLAR (PNATE)</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com a União, cuja destinação encontra-se vinculada a programas da educação.</t>
+          <t>Controle dos recursos originários de transferências do Fundo Nacional do Desenvolvimento da Educação - FNDE, destinados ao Programa Nacional de Apoio ao Transporte Escolar (PNATE).</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>571</v>
+        <v>569</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Transferências do Estado referentes a Convênios e Instrumentos Congêneres vinculados à Educação</t>
+          <t>OUTRAS TRANSFERÊNCIAS DE RECURSOS DO FNDE</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com os Estados, cuja destinação encontra-se vinculada a programas da educação.</t>
+          <t>Controle dos demais recursos originários de transferências do Fundo Nacional do Desenvolvimento da Educação - FNDE.</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17">
-        <v>572</v>
+        <v>570</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Transferências de Municípios referentes a Convênios e Instrumentos Congêneres vinculados à Educação</t>
+          <t>TRANSFERÊNCIAS DO GOVERNO FEDERAL REFERENTES A CONVÊNIOS E INSTRUMENTOS CONGÊNERES VINCULADOS À EDUCAÇÃO</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com outros municípios, cuja destinação encontra-se vinculada a programas da educação.</t>
+          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com a União, cuja destinação encontra-se vinculada a programas da educação.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18">
-        <v>573</v>
+        <v>571</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Royalties e Participação Especial de Petróleo e Gás Natural Vinculados à Educação - Lei nº 12.858/2013</t>
+          <t>TRANSFERÊNCIAS DO ESTADO REFERENTES A CONVÊNIOS E INSTRUMENTOS CONGÊNERES VINCULADOS À EDUCAÇÃO</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Controle dos recursos vinculados à Educação, originários de transferências recebidas pelos entes, relativos a Royalties e Participação Especial com base no art. 2º da Lei nº 12.858/2013.</t>
+          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com os Estados, cuja destinação encontra-se vinculada a programas da educação.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19">
-        <v>574</v>
+        <v>572</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Operações de Crédito Vinculadas à Educação</t>
+          <t>TRANSFERÊNCIAS DE MUNICÍPIOS REFERENTES A CONVÊNIOS E INSTRUMENTOS CONGÊNERES VINCULADOS À EDUCAÇÃO</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de operações de crédito, cuja destinação encontra-se vinculada a programas da educação.</t>
+          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com outros municípios, cuja destinação encontra-se vinculada a programas da educação.</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20">
-        <v>575</v>
+        <v>573</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Outras Transferências de Convênios e Instrumentos Congêneres vinculados à Educação</t>
+          <t>ROYALTIES E PARTICIPAÇÃO ESPECIAL DE PETRÓLEO E GÁS NATURAL VINCULADOS À EDUCAÇÃO - LEI Nº 12.858/2013</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências de entidades privadas, estrangeiras ou multigovernamentais em virtude de assinatura de convênios e instrumentos congêneres, cuja destinação encontra-se vinculada a programas de educação.</t>
+          <t>Controle dos recursos vinculados à Educação, originários de transferências recebidas pelos entes, relativos a Royalties e Participação Especial com base no art. 2º da Lei nº 12.858/2013.</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21">
-        <v>576</v>
+        <v>574</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Transferências de Recursos dos Estados para programas de educação</t>
+          <t>OPERAÇÕES DE CRÉDITO VINCULADAS À EDUCAÇÃO</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Controle dos recursos transferidos pelos Estados para programas de educação, que não decorram de celebração de convênios, contratos de repasse e termos de parceria.</t>
+          <t>Controle dos recursos originários de operações de crédito, cuja destinação encontra-se vinculada a programas da educação.</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22">
-        <v>599</v>
+        <v>575</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Outros Recursos Vinculados à Educação</t>
+          <t>OUTRAS TRANSFERÊNCIAS DE CONVÊNIOS E INSTRUMENTOS CONGÊNERES VINCULADOS À EDUCAÇÃO</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Controle dos demais recursos vinculados à Educação, não enquadrados nas especificações anteriores.</t>
+          <t>Controle dos recursos originários de transferências de entidades privadas, estrangeiras ou multigovernamentais em virtude de assinatura de convênios e instrumentos congêneres, cuja destinação encontra-se vinculada a programas de educação.</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23">
-        <v>600</v>
+        <v>576</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Transferências Fundo a Fundo de Recursos do SUS provenientes do Governo Federal - Bloco de Manutenção das Ações e Serviços Públicos de Saúde</t>
+          <t>TRANSFERÊNCIAS DE RECURSOS DOS ESTADOS PARA PROGRAMAS DE EDUCAÇÃO</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências do Fundo Nacional de Saúde, referentes ao Sistema Único de Saúde (SUS) e relacionados ao Bloco de Manutenção das Ações e Serviços Públicos de Saúde.</t>
+          <t>Controle dos recursos transferidos pelos Estados para programas de educação, que não decorram de celebração de convênios, contratos de repasse e termos de parceria.</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24">
-        <v>601</v>
+        <v>599</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Transferências Fundo a Fundo de Recursos do SUS provenientes do Governo Federal - Bloco de Estruturação da Rede de Serviços Públicos de Saúde</t>
+          <t>OUTROS RECURSOS VINCULADOS À EDUCAÇÃO</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências do Fundo Nacional de Saúde, referentes ao Sistema Único de Saúde (SUS) e relacionados ao Bloco de Estruturação na Rede de Serviços Públicos de Saúde.</t>
+          <t>Controle dos demais recursos vinculados à Educação, não enquadrados nas especificações anteriores.</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25">
-        <v>602</v>
+        <v>600</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Transferências Fundo a Fundo de Recursos do SUS provenientes do Governo Federal -  Bloco de Manutenção das Ações e Serviços Públicos de Saúde -  Recursos destinados ao enfrentamento da COVID-19 no bojo da ação 21C0.</t>
+          <t>TRANSFERÊNCIAS FUNDO A FUNDO DE RECURSOS DO SUS PROVENIENTES DO GOVERNO FEDERAL - BLOCO DE MANUTENÇÃO DAS AÇÕES E SERVIÇOS PÚBLICOS DE SAÚDE</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências do Fundo Nacional de Saúde, referentes ao Sistema Único de Saúde (SUS), relacionados ao Bloco de Manutenção das Ações e Serviços Públicos de Saúde, e destinados ao enfrentamento da COVID-19 no bojo da ação 21C0 do orçamento da União.</t>
+          <t>Controle dos recursos originários de transferências do Fundo Nacional de Saúde, referentes ao Sistema Único de Saúde (SUS) e relacionados ao Bloco de Manutenção das Ações e Serviços Públicos de Saúde.</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26">
-        <v>603</v>
+        <v>601</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Transferências Fundo a Fundo de Recursos do SUS provenientes do Governo Federal -  Bloco de Estruturação da Rede de Serviços Públicos de Saúde -  Recursos destinados ao enfrentamento da COVID-19 no bojo da ação 21C0.</t>
+          <t>TRANSFERÊNCIAS FUNDO A FUNDO DE RECURSOS DO SUS PROVENIENTES DO GOVERNO FEDERAL - BLOCO DE ESTRUTURAÇÃO DA REDE DE SERVIÇOS PÚBLICOS DE SAÚDE</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências do Fundo Nacional de Saúde, referentes ao Sistema Único de Saúde (SUS), relacionados ao Bloco de Estruturação na Rede de Serviços Públicos de Saúde e destinados ao enfrentamento da COVID-19 no bojo da ação 21C0 do orçamento da União.</t>
+          <t>Controle dos recursos originários de transferências do Fundo Nacional de Saúde, referentes ao Sistema Único de Saúde (SUS) e relacionados ao Bloco de Estruturação na Rede de Serviços Públicos de Saúde.</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27">
-        <v>604</v>
+        <v>602</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Transferências provenientes do Governo Federal destinadas ao vencimento dos agentes comunitários de saúde e dos agentes de combate às endemias</t>
+          <t>TRANSFERÊNCIAS FUNDO A FUNDO DE RECURSOS DO SUS PROVENIENTES DO GOVERNO FEDERAL -  BLOCO DE MANUTENÇÃO DAS AÇÕES E SERVIÇOS PÚBLICOS DE SAÚDE -  RECURSOS DESTINADOS AO ENFRENTAMENTO DA COVID-19 NO BOJO DA AÇÃO 21C0.</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários do Governo Federal, referentes ao Sistema Único de Saúde (SUS), relacionados ao vencimento dos agentes comunitários de saúde e dos agentes de combate às endemias, nos termos do art. 198, §7ª da Constituição Federal.</t>
+          <t>Controle dos recursos originários de transferências do Fundo Nacional de Saúde, referentes ao Sistema Único de Saúde (SUS), relacionados ao Bloco de Manutenção das Ações e Serviços Públicos de Saúde, e destinados ao enfrentamento da COVID-19 no bojo da ação 21C0 do orçamento da União.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28">
-        <v>605</v>
+        <v>603</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Assistência financeira da União destinada à complementação ao pagamento dos pisos salariais para profissionais da enfermagem.</t>
+          <t>TRANSFERÊNCIAS FUNDO A FUNDO DE RECURSOS DO SUS PROVENIENTES DO GOVERNO FEDERAL -  BLOCO DE ESTRUTURAÇÃO DA REDE DE SERVIÇOS PÚBLICOS DE SAÚDE -  RECURSOS DESTINADOS AO ENFRENTAMENTO DA COVID-19 NO BOJO DA AÇÃO 21C0.</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Controle dos recursos transferidos pela União, a título de assistência financeira complementar, para o cumprimento dos pisos salariais profissionais nacionais para o enfermeiro,  o técnico de enfermagem, o auxiliar de enfermagem e a parteira, conforme estabelecido pela CF/88, art. 198, §§12 a 15.</t>
+          <t>Controle dos recursos originários de transferências do Fundo Nacional de Saúde, referentes ao Sistema Único de Saúde (SUS), relacionados ao Bloco de Estruturação na Rede de Serviços Públicos de Saúde e destinados ao enfrentamento da COVID-19 no bojo da ação 21C0 do orçamento da União.</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29">
-        <v>621</v>
+        <v>604</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Transferências Fundo a Fundo de Recursos do SUS provenientes do Governo Estadual</t>
+          <t>TRANSFERÊNCIAS PROVENIENTES DO GOVERNO FEDERAL DESTINADAS AO VENCIMENTO DOS AGENTES COMUNITÁRIOS DE SAÚDE E DOS AGENTES DE COMBATE ÀS ENDEMIAS</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências do Fundo Estadual de Saúde, referentes ao Sistema Único de Saúde (SUS).</t>
+          <t>Controle dos recursos originários do Governo Federal, referentes ao Sistema Único de Saúde (SUS), relacionados ao vencimento dos agentes comunitários de saúde e dos agentes de combate às endemias, nos termos do art. 198, §7ª da Constituição Federal.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30">
-        <v>622</v>
+        <v>605</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Transferências Fundo a Fundo de Recursos do SUS provenientes dos Governos Municipais</t>
+          <t>ASSISTÊNCIA FINANCEIRA DA UNIÃO DESTINADA À COMPLEMENTAÇÃO AO PAGAMENTO DOS PISOS SALARIAIS PARA PROFISSIONAIS DA ENFERMAGEM.</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências dos Fundos de Saúde de outros municípios, referentes ao Sistema Único de Saúde (SUS).</t>
+          <t>Controle dos recursos transferidos pela União, a título de assistência financeira complementar, para o cumprimento dos pisos salariais profissionais nacionais para o enfermeiro,  o técnico de enfermagem, o auxiliar de enfermagem e a parteira, conforme estabelecido pela CF/88, art. 198, §§12 a 15.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31">
-        <v>631</v>
+        <v>621</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Transferências do Governo Federal referentes a Convênios e Instrumentos Congêneres vinculados à Saúde</t>
+          <t>TRANSFERÊNCIAS FUNDO A FUNDO DE RECURSOS DO SUS PROVENIENTES DO GOVERNO ESTADUAL</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com a União, cuja destinação encontra-se vinculada a programas da saúde.</t>
+          <t>Controle dos recursos originários de transferências do Fundo Estadual de Saúde, referentes ao Sistema Único de Saúde (SUS).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32">
-        <v>632</v>
+        <v>622</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Transferências do Estado referentes a Convênios e Instrumentos Congêneres vinculados à Saúde</t>
+          <t>TRANSFERÊNCIAS FUNDO A FUNDO DE RECURSOS DO SUS PROVENIENTES DOS GOVERNOS MUNICIPAIS</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com os Estados, cuja destinação encontra-se vinculada a programas da saúde.</t>
+          <t>Controle dos recursos originários de transferências dos Fundos de Saúde de outros municípios, referentes ao Sistema Único de Saúde (SUS).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33">
-        <v>633</v>
+        <v>631</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Transferências de Municípios referentes a Convênios Instrumentos Congêneres vinculados à Saúde</t>
+          <t>TRANSFERÊNCIAS DO GOVERNO FEDERAL REFERENTES A CONVÊNIOS E INSTRUMENTOS CONGÊNERES VINCULADOS À SAÚDE</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com outros Municípios, cuja destinação encontra-se vinculada a programas da saúde.</t>
+          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com a União, cuja destinação encontra-se vinculada a programas da saúde.</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34">
-        <v>634</v>
+        <v>632</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Operações de Crédito vinculadas à Saúde</t>
+          <t>TRANSFERÊNCIAS DO ESTADO REFERENTES A CONVÊNIOS E INSTRUMENTOS CONGÊNERES VINCULADOS À SAÚDE</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de operações de crédito, cuja destinação encontra-se vinculada a programas da saúde.</t>
+          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com os Estados, cuja destinação encontra-se vinculada a programas da saúde.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35">
-        <v>635</v>
+        <v>633</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Royalties e Participação Especial de Petróleo e Gás Natural vinculados à Saúde - Lei nº 12.858/2013</t>
+          <t>TRANSFERÊNCIAS DE MUNICÍPIOS REFERENTES A CONVÊNIOS INSTRUMENTOS CONGÊNERES VINCULADOS À SAÚDE</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Controle dos recursos vinculados à Saúde, originários de transferências recebidas pelos entes, relativos a Royalties e Participação Especial com base no art. 2º  da Lei nº 12.858/2013.</t>
+          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres com outros Municípios, cuja destinação encontra-se vinculada a programas da saúde.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36">
-        <v>636</v>
+        <v>634</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Outras Transferências de Convênios e Instrumentos Congêneres vinculados à Saúde</t>
+          <t>OPERAÇÕES DE CRÉDITO VINCULADAS À SAÚDE</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências de entidades privadas, estrangeiras ou multigovernamentais em virtude de assinatura de convênios e instrumentos congêneres, cuja destinação encontra-se vinculada a programas de saúde.</t>
+          <t>Controle dos recursos originários de operações de crédito, cuja destinação encontra-se vinculada a programas da saúde.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37">
-        <v>659</v>
+        <v>635</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Outros Recursos Vinculados à Saúde</t>
+          <t>ROYALTIES E PARTICIPAÇÃO ESPECIAL DE PETRÓLEO E GÁS NATURAL VINCULADOS À SAÚDE - LEI Nº 12.858/2013</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Controle dos demais recursos vinculados à Saúde, não enquadrados nas especificações anteriores.</t>
+          <t>Controle dos recursos vinculados à Saúde, originários de transferências recebidas pelos entes, relativos a Royalties e Participação Especial com base no art. 2º  da Lei nº 12.858/2013.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38">
-        <v>660</v>
+        <v>636</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Transferência de Recursos do Fundo Nacional de Assistência Social - FNAS</t>
+          <t>OUTRAS TRANSFERÊNCIAS DE CONVÊNIOS E INSTRUMENTOS CONGÊNERES VINCULADOS À SAÚDE</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Controle os recursos originários de transferências do Fundo Nacional de Assistência Social - Lei Federal nº 8.742, 07/12/1993.</t>
+          <t>Controle dos recursos originários de transferências de entidades privadas, estrangeiras ou multigovernamentais em virtude de assinatura de convênios e instrumentos congêneres, cuja destinação encontra-se vinculada a programas de saúde.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39">
-        <v>661</v>
+        <v>659</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Transferência de Recursos dos Fundos Estaduais de Assistência Social</t>
+          <t>OUTROS RECURSOS VINCULADOS À SAÚDE</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências dos fundos estaduais de assistência social.</t>
+          <t>Controle dos demais recursos vinculados à Saúde, não enquadrados nas especificações anteriores.</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40">
-        <v>662</v>
+        <v>660</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Transferências de Recursos dos Fundos Municipais de Assistência Social</t>
+          <t>TRANSFERÊNCIA DE RECURSOS DO FUNDO NACIONAL DE ASSISTÊNCIA SOCIAL - FNAS</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Controle os recursos originários de transferência dos fundos municipais de assistência social.</t>
+          <t>Controle os recursos originários de transferências do Fundo Nacional de Assistência Social - Lei Federal nº 8.742, 07/12/1993.</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41">
-        <v>665</v>
+        <v>661</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Transferências de Convênios e Instrumentos Congêneres vinculados à Assistência Social</t>
+          <t>TRANSFERÊNCIA DE RECURSOS DOS FUNDOS ESTADUAIS DE ASSISTÊNCIA SOCIAL</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres cuja destinação encontra-se vinculada a programas da assistência social.</t>
+          <t>Controle dos recursos originários de transferências dos fundos estaduais de assistência social.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42">
-        <v>669</v>
+        <v>662</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Outros Recursos Vinculados à Assistência Social</t>
+          <t>TRANSFERÊNCIAS DE RECURSOS DOS FUNDOS MUNICIPAIS DE ASSISTÊNCIA SOCIAL</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Controle dos demais recursos vinculados à Assistência Social, não enquadrados nas especificações anteriores.</t>
+          <t>Controle os recursos originários de transferência dos fundos municipais de assistência social.</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43">
-        <v>700</v>
+        <v>665</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Outras Transferências de Convênios ou Instrumentos Congêneres da União</t>
+          <t>TRANSFERÊNCIAS DE CONVÊNIOS E INSTRUMENTOS CONGÊNERES VINCULADOS À ASSISTÊNCIA SOCIAL</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências federais em decorrência da celebração de convênios e instrumentos congêneres cuja destinação encontra-se vinculada aos seus objetos. Não serão controlados por esta fonte os recursos de convênios vinculados a programas da educação, da saúde e da assistência social.</t>
+          <t>Controle dos recursos originários de transferências em decorrência da celebração de convênios e instrumentos congêneres cuja destinação encontra-se vinculada a programas da assistência social.</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44">
-        <v>701</v>
+        <v>669</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Outras Transferências de Convênios ou Instrumentos Congêneres dos Estados</t>
+          <t>OUTROS RECURSOS VINCULADOS À ASSISTÊNCIA SOCIAL</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências estaduais em decorrência da celebração de convênios e instrumentos congêneres, cuja destinação encontra-se vinculada aos seus objetos. Não serão controlados por esta fonte os recursos de convênios ou contratos de repasse vinculados a programas da educação, da saúde e da assistência social.</t>
+          <t>Controle dos demais recursos vinculados à Assistência Social, não enquadrados nas especificações anteriores.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45">
-        <v>702</v>
+        <v>700</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Outras Transferências de Convênios ou Instrumentos Congêneres dos Municípios</t>
+          <t>OUTRAS TRANSFERÊNCIAS DE CONVÊNIOS OU INSTRUMENTOS CONGÊNERES DA UNIÃO</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências de municípios em decorrência da celebração de convênios e instrumentos congêneres, cuja destinação encontra-se vinculada aos seus objetos. Não serão controlados por esta fonte os recursos de convênios ou contratos de repasse vinculados a programas da educação, da saúde e da assistência social.</t>
+          <t>Controle dos recursos originários de transferências federais em decorrência da celebração de convênios e instrumentos congêneres cuja destinação encontra-se vinculada aos seus objetos. Não serão controlados por esta fonte os recursos de convênios vinculados a programas da educação, da saúde e da assistência social.</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46">
-        <v>703</v>
+        <v>701</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Outras Transferências de Convênios ou Instrumentos Congêneres de outras Entidades</t>
+          <t>OUTRAS TRANSFERÊNCIAS DE CONVÊNIOS OU INSTRUMENTOS CONGÊNERES DOS ESTADOS</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de transferências de entidades privadas, estrangeiras ou multigovernamentais em virtude de assinatura de convênios e instrumentos congêneres, cuja destinação encontra-se vinculada aos seus objetos. Não serão controlados por esta fonte os recursos de convênios ou contratos de repasse vinculados a programas da educação, da saúde e da assistência social.</t>
+          <t>Controle dos recursos originários de transferências estaduais em decorrência da celebração de convênios e instrumentos congêneres, cuja destinação encontra-se vinculada aos seus objetos. Não serão controlados por esta fonte os recursos de convênios ou contratos de repasse vinculados a programas da educação, da saúde e da assistência social.</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47">
-        <v>705</v>
+        <v>702</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Transferências dos Estados Referentes a Compensações Financeiras pela Exploração de Recursos Naturais</t>
+          <t>OUTRAS TRANSFERÊNCIAS DE CONVÊNIOS OU INSTRUMENTOS CONGÊNERES DOS MUNICÍPIOS</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Controle dos recursos transferidos pelos Estados, originários da arrecadação de royalties do petróleo, do gás natural, da cota-parte do bônus de assinatura de contrato de partilha de produção.</t>
+          <t>Controle dos recursos originários de transferências de municípios em decorrência da celebração de convênios e instrumentos congêneres, cuja destinação encontra-se vinculada aos seus objetos. Não serão controlados por esta fonte os recursos de convênios ou contratos de repasse vinculados a programas da educação, da saúde e da assistência social.</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48">
-        <v>706</v>
+        <v>703</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Transferência Especial da União</t>
+          <t>OUTRAS TRANSFERÊNCIAS DE CONVÊNIOS OU INSTRUMENTOS CONGÊNERES DE OUTRAS ENTIDADES</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Controle dos recursos transferidos pela União provenientes de emendas individuais impositivas ao orçamento da União, por meio de transferências especiais, nos termos do art. 166-A da Constituição Federal.</t>
+          <t>Controle dos recursos originários de transferências de entidades privadas, estrangeiras ou multigovernamentais em virtude de assinatura de convênios e instrumentos congêneres, cuja destinação encontra-se vinculada aos seus objetos. Não serão controlados por esta fonte os recursos de convênios ou contratos de repasse vinculados a programas da educação, da saúde e da assistência social.</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49">
-        <v>707</v>
+        <v>704</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Transferências da União - inciso I do art. 5º da Lei Complementar 173/2020</t>
+          <t>TRANSFERÊNCIAS DA UNIÃO REFERENTES A COMPENSAÇÕES FINANCEIRAS PELA EXPLORAÇÃO DE RECURSOS NATURAIS</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Controle dos recursos provenientes de transferência da União com base no disposto no inciso I do art. 5º da Lei Complementar 173, de 27 de maio de 2020.</t>
+          <t>Controle dos recursos transferidos pela União, originários da arrecadação de royalties do petróleo, do gás natural, da cota-parte do bônus de assinatura de contrato de partilha de produção, exceto os recursos provenientes da Lei nº 12.858/2013, destinados às áreas da saúde ou da educação.</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50">
-        <v>708</v>
+        <v>705</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Transferência da União Referente à Compensação Financeira de Recursos Minerais</t>
+          <t>TRANSFERÊNCIAS DOS ESTADOS REFERENTES A COMPENSAÇÕES FINANCEIRAS PELA EXPLORAÇÃO DE RECURSOS NATURAIS</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Controle dos recursos transferidos pela União, referentes à compensação financeira pela exploração de recursos minerais em atendimento às destinações e vedações previstas na legislação.</t>
+          <t>Controle dos recursos transferidos pelos Estados, originários da arrecadação de royalties do petróleo, do gás natural, da cota-parte do bônus de assinatura de contrato de partilha de produção.</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51">
-        <v>709</v>
+        <v>706</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Transferência da União referente à Compensação Financeira de Recursos Hídricos</t>
+          <t>TRANSFERÊNCIA ESPECIAL DA UNIÃO</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Controle dos recursos transferidos pela União, referentes à compensação financeira de recursos hídricos em atendimento às destinações e vedações previstas na legislação.</t>
+          <t>Controle dos recursos transferidos pela União provenientes de emendas individuais impositivas ao orçamento da União, por meio de transferências especiais, nos termos do art. 166-A da Constituição Federal.</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52">
-        <v>710</v>
+        <v>707</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Transferência Especial dos Estados</t>
+          <t>TRANSFERÊNCIAS DA UNIÃO - INCISO I DO ART. 5º DA LEI COMPLEMENTAR 173/2020</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Controle dos recursos transferidos pelos Estados provenientes de emendas individuais impositivas ao orçamento desses entes, por meio de transferências especiais, nos termos das constituições estaduais que reproduziram o disposto no art. 166-A da Constituição Federal.</t>
+          <t>Controle dos recursos provenientes de transferência da União com base no disposto no inciso I do art. 5º da Lei Complementar 173, de 27 de maio de 2020.</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53">
-        <v>711</v>
+        <v>708</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Demais Transferências Obrigatórias não Decorrentes de Repartições de Receitas.</t>
+          <t>TRANSFERÊNCIA DA UNIÃO REFERENTE À COMPENSAÇÃO FINANCEIRA DE RECURSOS MINERAIS</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Controla os recursos originários de transferências obrigatórias da União que não decorram de repartição de receitas, como as transferências a título de auxílio ou apoio financeiro, e para os quais não tenha sido criada fonte ou destinação de receitas específica.</t>
+          <t>Controle dos recursos transferidos pela União, referentes à compensação financeira pela exploração de recursos minerais em atendimento às destinações e vedações previstas na legislação.</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54">
-        <v>712</v>
+        <v>709</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Transferências Fundo a Fundo de Recursos do Fundo Penitenciário - FUNPEN</t>
+          <t>TRANSFERÊNCIA DA UNIÃO REFERENTE À COMPENSAÇÃO FINANCEIRA DE RECURSOS HÍDRICOS</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Controla as transferências obrigatórias de recursos do Fundo Penitenciário Nacional - FUNPEN.</t>
+          <t>Controle dos recursos transferidos pela União, referentes à compensação financeira de recursos hídricos em atendimento às destinações e vedações previstas na legislação.</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55">
-        <v>713</v>
+        <v>710</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Transferências Fundo a Fundo de Recursos do Fundo de Segurança Pública - FSP</t>
+          <t>TRANSFERÊNCIA ESPECIAL DOS ESTADOS</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Controla as transferências obrigatórias de recursos do Fundo de Segurança Pública - FSP</t>
+          <t>Controle dos recursos transferidos pelos Estados provenientes de emendas individuais impositivas ao orçamento desses entes, por meio de transferências especiais, nos termos das constituições estaduais que reproduziram o disposto no art. 166-A da Constituição Federal.</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56">
-        <v>714</v>
+        <v>711</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Transferências Fundo a Fundo de Recursos do Fundo de Amparo ao Trabalhador - FAT</t>
+          <t>DEMAIS TRANSFERÊNCIAS OBRIGATÓRIAS NÃO DECORRENTES DE REPARTIÇÕES DE RECEITAS.</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Controla as transferências obrigatórias de recursos do Fundo de Amparo ao Trabalhador - FAT</t>
+          <t>Controla os recursos originários de transferências obrigatórias da União que não decorram de repartição de receitas, como as transferências a título de auxílio ou apoio financeiro, e para os quais não tenha sido criada fonte ou destinação de receitas específica.</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57">
-        <v>715</v>
+        <v>712</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Transferências Destinadas ao Setor Cultural - LC nº 195/2022 - Art. 5º - Audiovisual</t>
+          <t>TRANSFERÊNCIAS FUNDO A FUNDO DE RECURSOS DO FUNDO PENITENCIÁRIO - FUNPEN</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Controla a parcela dos recursos provenientes das transferências efetuadas pela União destinadas ao setor cultural, especificamente ao setor audiovisual, como ação emergencial adotada em decorrência dos efeitos econômicos e sociais da pandemia da covid-19, em cumprimento ao Art. 5º da Lei Complementar nº 195, de 8 de julho de 2022.</t>
+          <t>Controla as transferências obrigatórias de recursos do Fundo Penitenciário Nacional - FUNPEN.</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58">
-        <v>716</v>
+        <v>713</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Transferências Destinadas ao Setor cultural - LC nº 195/2022 - Art. 8º - Demais Setores da Cultura</t>
+          <t>TRANSFERÊNCIAS FUNDO A FUNDO DE RECURSOS DO FUNDO DE SEGURANÇA PÚBLICA - FSP</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Controla a parcela dos recursos provenientes das transferências efetuadas pela União destinadas ao setor cultural, como ação emergencial adotada em decorrência dos efeitos econômicos e sociais da pandemia da covid-19, em cumprimento ao Art. 8º da Lei Complementar nº 195, de 8 de julho de 2022</t>
+          <t>Controla as transferências obrigatórias de recursos do Fundo de Segurança Pública - FSP</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59">
-        <v>717</v>
+        <v>714</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Assistência Financeira Transporte Coletivo - Art. 5º, Inciso IV, EC nº 123/2022</t>
+          <t>TRANSFERÊNCIAS FUNDO A FUNDO DE RECURSOS DO FUNDO DE AMPARO AO TRABALHADOR - FAT</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Controla os recursos provenientes das transferências da União a título de assistência financeira a serem utilizados no custeio da garantia prevista no §2º do art. 230 da CF, de gratuidade dos transportes coletivos urbanos aos maiores de 65 anos, conforme prevê o inciso IV, art. 5º, da Emenda Constitucional nº 123/2022.</t>
+          <t>Controla as transferências obrigatórias de recursos do Fundo de Amparo ao Trabalhador - FAT</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60">
-        <v>718</v>
+        <v>715</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Auxílio Financeiro - Outorga Crédito Tributário ICMS - Art. 5º, Inciso V, EC nº 123/2022</t>
+          <t>TRANSFERÊNCIAS DESTINADAS AO SETOR CULTURAL - LC Nº 195/2022 - ART. 5º - AUDIOVISUAL</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Controla os recursos provenientes das transferências da União a título de auxílio financeiro para os Estados e o Distrito Federal que outorgarem créditos tributários do Imposto sobre Operações relativas à Circulação de Mercadorias e sobre Prestações de Serviços de Transporte Interestadual e Intermunicipal e de Comunicação (ICMS) aos produtores ou distribuidores de etanol hidratado em seu território, em montante equivalente ao valor recebido, conforme prevê o Inciso V, art. 5º, da Emenda Constitucional nº 123/2022.</t>
+          <t>Controla a parcela dos recursos provenientes das transferências efetuadas pela União destinadas ao setor cultural, especificamente ao setor audiovisual, como ação emergencial adotada em decorrência dos efeitos econômicos e sociais da pandemia da covid-19, em cumprimento ao Art. 5º da Lei Complementar nº 195, de 8 de julho de 2022.</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61">
-        <v>719</v>
+        <v>716</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Transferências da Política Nacional Aldir Blanc de Fomento à Cultura - Lei nº 14.399/2022</t>
+          <t>TRANSFERÊNCIAS DESTINADAS AO SETOR CULTURAL - LC Nº 195/2022 - ART. 8º - DEMAIS SETORES DA CULTURA</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Controla os recursos provenientes de transferências efetuadas pela União em decorrência da Política Nacional Aldir Blanc de Fomento à Cultura previstas no art. 6º da Lei nº 14.399, de 8 de julho de 2022.</t>
+          <t>Controla a parcela dos recursos provenientes das transferências efetuadas pela União destinadas ao setor cultural, como ação emergencial adotada em decorrência dos efeitos econômicos e sociais da pandemia da covid-19, em cumprimento ao Art. 8º da Lei Complementar nº 195, de 8 de julho de 2022</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62">
-        <v>720</v>
+        <v>717</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Transferências da União Referentes às participações na exploração de Petróleo e Gás Natural destinadas ao FEP - Lei 9.478/1997</t>
+          <t>ASSISTÊNCIA FINANCEIRA TRANSPORTE COLETIVO - ART. 5º, INCISO IV, EC Nº 123/2022</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Transferências da União referentes às participações na exploração de petróleo, gás natural e outros hidrocarbonetos fluidos,  destinadas ao Fundo Especial - FEP, conforme estabelece o art. 50-F da Lei 9.478/97,  exceto os recursos obrigatórios para educação e saúde de que trata a Lei 12.858/2013.</t>
+          <t>Controla os recursos provenientes das transferências da União a título de assistência financeira a serem utilizados no custeio da garantia prevista no §2º do art. 230 da CF, de gratuidade dos transportes coletivos urbanos aos maiores de 65 anos, conforme prevê o inciso IV, art. 5º, da Emenda Constitucional nº 123/2022.</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63">
-        <v>721</v>
+        <v>718</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Transferências da União Referentes a Cessão Onerosa de Petróleo - Lei nº 13.885/2019</t>
+          <t>AUXÍLIO FINANCEIRO - OUTORGA CRÉDITO TRIBUTÁRIO ICMS - ART. 5º, INCISO V, EC Nº 123/2022</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Controle dos recursos transferidos pela União, provenientes da cessão onerosa à Petróleo Brasileiro S.A. - PETROBRAS,  do exercício das atividades de pesquisa e lavra de petróleo, gás natural e outros hidrocarbonetos fluidos,  originários dos leilões dos volumes excedentes ao limite a que se refere o § 2º do art. 1º da Lei nº 12.276,  conforme estabelecido na Lei nº 13.885/2019.</t>
+          <t>Controla os recursos provenientes das transferências da União a título de auxílio financeiro para os Estados e o Distrito Federal que outorgarem créditos tributários do Imposto sobre Operações relativas à Circulação de Mercadorias e sobre Prestações de Serviços de Transporte Interestadual e Intermunicipal e de Comunicação (ICMS) aos produtores ou distribuidores de etanol hidratado em seu território, em montante equivalente ao valor recebido, conforme prevê o Inciso V, art. 5º, da Emenda Constitucional nº 123/2022.</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64">
-        <v>749</v>
+        <v>719</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Outras vinculações de transferências</t>
+          <t>TRANSFERÊNCIAS DA POLÍTICA NACIONAL ALDIR BLANC DE FOMENTO À CULTURA - LEI Nº 14.399/2022</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Controle dos recursos de outras transferências vinculadas, não enquadrados nas especificações anteriores.</t>
+          <t>Controla os recursos provenientes de transferências efetuadas pela União em decorrência da Política Nacional Aldir Blanc de Fomento à Cultura previstas no art. 6º da Lei nº 14.399, de 8 de julho de 2022.</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65">
-        <v>750</v>
+        <v>720</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Recursos da Contribuição de Intervenção no Domínio Econômico - CIDE</t>
+          <t>TRANSFERÊNCIAS DA UNIÃO REFERENTES ÀS PARTICIPAÇÕES NA EXPLORAÇÃO DE PETRÓLEO E GÁS NATURAL DESTINADAS AO FEP - LEI 9.478/1997</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Controle dos recursos recebidos pelos Estados, Distrito Federal e Municípios, decorrentes da distribuição da arrecadação da União com a CIDE - Combustíveis, com base no disposto na Lei nº 10.336/2001.</t>
+          <t>Transferências da União referentes às participações na exploração de petróleo, gás natural e outros hidrocarbonetos fluidos,  destinadas ao Fundo Especial - FEP, conforme estabelece o art. 50-F da Lei 9.478/97,  exceto os recursos obrigatórios para educação e saúde de que trata a Lei 12.858/2013.</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66">
-        <v>751</v>
+        <v>721</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Recursos da Contribuição para o Custeio do Serviço de Iluminação Pública - COSIP</t>
+          <t>TRANSFERÊNCIAS DA UNIÃO REFERENTES A CESSÃO ONEROSA DE PETRÓLEO - LEI Nº 13.885/2019</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Controle dos recursos da COSIP, nos termos do artigo 149-A da Constituição Federal da República.</t>
+          <t>Controle dos recursos transferidos pela União, provenientes da cessão onerosa à Petróleo Brasileiro S.A. - PETROBRAS,  do exercício das atividades de pesquisa e lavra de petróleo, gás natural e outros hidrocarbonetos fluidos,  originários dos leilões dos volumes excedentes ao limite a que se refere o § 2º do art. 1º da Lei nº 12.276,  conforme estabelecido na Lei nº 13.885/2019.</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67">
-        <v>752</v>
+        <v>747</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Recursos Vinculados ao Trânsito</t>
+          <t>OUTRAS VINCULAÇÕES DE TRANSFERÊNCIAS DA UNIÃO</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Controle dos recursos com a cobrança das multas de trânsito nos termos do art. 320 da Lei nº 9.503/1997 - Código de Trânsito Brasileiro.</t>
+          <t>Controle dos recursos de outras transferências vinculadas da União, não enquadrados nas  especificações anteriores.</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68">
-        <v>753</v>
+        <v>748</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Recursos Provenientes de Taxas, Contribuições e Preços Públicos</t>
+          <t>OUTRAS VINCULAÇÕES DE TRANSFERÊNCIAS DOS ESTADOS</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Controle dos recursos de taxas, contribuições e preços públicos vinculados conforme legislações específicas.</t>
+          <t>Controle dos recursos de outras transferências vinculadas dos Estados, não enquadrados nas  especificações anteriores.</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69">
-        <v>754</v>
+        <v>749</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Recursos de Operações de Crédito</t>
+          <t>OUTRAS VINCULAÇÕES DE TRANSFERÊNCIAS</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Controle dos recursos originários de operações de crédito, exceto as operações cuja aplicação esteja destinada a programas de educação e saúde.</t>
+          <t>Controle dos recursos de outras transferências vinculadas, não enquadrados nas especificações anteriores.</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70">
-        <v>755</v>
+        <v>750</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Recursos de Alienação de Bens/Ativos - Administração Direta</t>
+          <t>RECURSOS DA CONTRIBUIÇÃO DE INTERVENÇÃO NO DOMÍNIO ECONÔMICO - CIDE</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Controle dos recursos decorrentes da alienação de bens da Administração Direta, nos termos do art. 44 da Lei Complementar nº 101/2000.</t>
+          <t>Controle dos recursos recebidos pelos Estados, Distrito Federal e Municípios, decorrentes da distribuição da arrecadação da União com a CIDE - Combustíveis, com base no disposto na Lei nº 10.336/2001.</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71">
-        <v>756</v>
+        <v>751</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Recursos de Alienação de Bens/Ativos - Administração Indireta</t>
+          <t>RECURSOS DA CONTRIBUIÇÃO PARA O CUSTEIO DO SERVIÇO DE ILUMINAÇÃO PÚBLICA - COSIP</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Controle dos recursos decorrentes da alienação de bens da Administração Indireta, nos termos do art. 44 da Lei Complementar nº 101/2000.</t>
+          <t>Controle dos recursos da COSIP, nos termos do artigo 149-A da Constituição Federal da República.</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72">
-        <v>757</v>
+        <v>752</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Recursos de Depósitos Judiciais - Lides das quais o Ente faz parte</t>
+          <t>RECURSOS VINCULADOS AO TRÂNSITO</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Controle dos recursos de depósitos judiciais apropriados pelo ente de lides das quais o ente faz parte, com base na Lei Complementar nº 151/2015, no art. 101 do ADCT da Constituição Federal.</t>
+          <t>Controle dos recursos com a cobrança das multas de trânsito nos termos do art. 320 da Lei nº 9.503/1997 - Código de Trânsito Brasileiro.</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73">
-        <v>758</v>
+        <v>753</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Recursos de Depósitos Judiciais - Lides das quais o Ente não faz parte</t>
+          <t>RECURSOS PROVENIENTES DE TAXAS, CONTRIBUIÇÕES E PREÇOS PÚBLICOS</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Controle dos recursos de depósitos judiciais apropriados pelo ente de lides das quais o ente não faz parte, com base no art. 101 do ADCT da Constituição Federal.</t>
+          <t>Controle dos recursos de taxas, contribuições e preços públicos vinculados conforme legislações específicas.</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74">
-        <v>759</v>
+        <v>754</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Recursos Vinculados a Fundos</t>
+          <t>RECURSOS DE OPERAÇÕES DE CRÉDITO</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Controle dos recursos vinculados a fundos, com exceção dos fundos relacionados à saúde, à educação, à assistência social e aos regimes de previdência.</t>
+          <t>Controle dos recursos originários de operações de crédito, exceto as operações cuja aplicação esteja destinada a programas de educação e saúde.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75">
-        <v>760</v>
+        <v>755</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Recursos de Emolumentos, Taxas e Custas</t>
+          <t>RECURSOS DE ALIENAÇÃO DE BENS/ATIVOS - ADMINISTRAÇÃO DIRETA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Controle dos recursos de emolumentos, taxas e outros recursos arrecadados, judiciais ou extrajudiciais, observado o disposto em legislações específicas.</t>
+          <t>Controle dos recursos decorrentes da alienação de bens da Administração Direta, nos termos do art. 44 da Lei Complementar nº 101/2000.</t>
         </is>
       </c>
     </row>
     <row r="76">
       <c r="A76">
-        <v>761</v>
+        <v>756</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Recursos Vinculados ao Fundo de Combate e Erradicação da Pobreza</t>
+          <t>RECURSOS DE ALIENAÇÃO DE BENS/ATIVOS - ADMINISTRAÇÃO INDIRETA</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Controle dos recursos vinculados ao Fundo de Combate e Erradicação da Pobreza, na forma prevista nos art. 82 do ADCT e da Lei Complementar nº 111, de 6 de julho de 2001.</t>
+          <t>Controle dos recursos decorrentes da alienação de bens da Administração Indireta, nos termos do art. 44 da Lei Complementar nº 101/2000.</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77">
-        <v>799</v>
+        <v>757</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Outras Vinculações Legais</t>
+          <t>RECURSOS DE DEPÓSITOS JUDICIAIS - LIDES DAS QUAIS O ENTE FAZ PARTE</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Controle de outros recursos vinculados por lei, não enquadrados nas especificações anteriores.</t>
+          <t>Controle dos recursos de depósitos judiciais apropriados pelo ente de lides das quais o ente faz parte, com base na Lei Complementar nº 151/2015, no art. 101 do ADCT da Constituição Federal.</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78">
-        <v>800</v>
+        <v>758</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Recursos Vinculados ao RPPS - Fundo em Capitalização (Plano Previdenciário)</t>
+          <t>RECURSOS DE DEPÓSITOS JUDICIAIS - LIDES DAS QUAIS O ENTE NÃO FAZ PARTE</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Controle dos recursos vinculados ao fundo em capitalização do RPPS. Esse plano existe tanto nos entes que segregaram quanto nos que não segregaram a massa dos segurados, observando-se o disposto na Portaria MF nº 464/2018. Na fase das despesas, será necessário associar esta fonte ao marcador que identifica a qual Poder ou Órgão se refere a despesa quando ela é executada no PO RPPS.</t>
+          <t>Controle dos recursos de depósitos judiciais apropriados pelo ente de lides das quais o ente não faz parte, com base no art. 101 do ADCT da Constituição Federal.</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79">
-        <v>801</v>
+        <v>759</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Recursos Vinculados ao RPPS - Fundo em Repartição (Plano Financeiro)</t>
+          <t>RECURSOS VINCULADOS A FUNDOS</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Controle dos recursos vinculados ao fundo em repartição do RPPS. Esse plano deve existir somente nos entes que segregaram a massa dos segurados, observando-se o disposto na Portaria MF nº 464/2018. Na fase da despesa, será necessário associar esta fonte ao marcador que identifica a qual Poder ou Órgão se refere a despesa quando ela é executada no PO RPPS.</t>
+          <t>Controle dos recursos vinculados a fundos, com exceção dos fundos relacionados à saúde, à educação, à assistência social e aos regimes de previdência.</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80">
-        <v>802</v>
+        <v>760</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Recursos Vinculados ao RPPS - Taxa de Administração</t>
+          <t>RECURSOS DE EMOLUMENTOS, TAXAS E CUSTAS</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Controle dos recursos destinados ao custeio das despesas necessárias à organização e ao funcionamento da unidade gestora do RPPS, observando-se o disposto na Portaria MPS nº 402/2008 e na Portaria MF nº 464/2018, ambas alteradas pela Portaria ME nº 19.451/2020.</t>
+          <t>Controle dos recursos de emolumentos, taxas e outros recursos arrecadados, judiciais ou extrajudiciais, observado o disposto em legislações específicas.</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81">
-        <v>803</v>
+        <v>761</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Recursos Vinculados ao Sistema de Proteção Social dos Militares (SPSM)</t>
+          <t>RECURSOS VINCULADOS AO FUNDO DE COMBATE E ERRADICAÇÃO DA POBREZA</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Controle dos recursos vinculados ao Sistema de Proteção Social dos Militares (SPSM), com base na Lei nº 6.880/1980 (Estatuto dos Militares), alterada pela Lei nº 13.954/2019.</t>
+          <t>Controle dos recursos vinculados ao Fundo de Combate e Erradicação da Pobreza, na forma prevista nos art. 82 do ADCT e da Lei Complementar nº 111, de 6 de julho de 2001.</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82">
-        <v>860</v>
+        <v>799</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Recursos Extraorçamentários Vinculados a Precatórios</t>
+          <t>OUTRAS VINCULAÇÕES LEGAIS</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Controle dos recursos financeiros junto aos tribunais de justiça vinculados ao pagamento de precatórios.</t>
+          <t>Controle de outros recursos vinculados por lei, não enquadrados nas especificações anteriores.</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83">
-        <v>861</v>
+        <v>800</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Recursos Extraorçamentários Vinculados a Depósitos Judiciais</t>
+          <t>RECURSOS VINCULADOS AO RPPS - FUNDO EM CAPITALIZAÇÃO (PLANO PREVIDENCIÁRIO)</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Controle dos recursos financeiros junto aos tribunais de justiça vinculados aos depósitos judiciais.</t>
+          <t>Controle dos recursos vinculados ao fundo em capitalização do RPPS. Esse plano existe tanto nos entes que segregaram quanto nos que não segregaram a massa dos segurados, observando-se o disposto na Portaria MF nº 464/2018. Na fase das despesas, será necessário associar esta fonte ao marcador que identifica a qual Poder ou Órgão se refere a despesa quando ela é executada no PO RPPS.</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84">
-        <v>862</v>
+        <v>801</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Recursos de Depósitos de Terceiros</t>
+          <t>RECURSOS VINCULADOS AO RPPS - FUNDO EM REPARTIÇÃO (PLANO FINANCEIRO)</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Controle dos recursos financeiros decorrentes de depósitos de terceiros.</t>
+          <t>Controle dos recursos vinculados ao fundo em repartição do RPPS. Esse plano deve existir somente nos entes que segregaram a massa dos segurados, observando-se o disposto na Portaria MF nº 464/2018. Na fase da despesa, será necessário associar esta fonte ao marcador que identifica a qual Poder ou Órgão se refere a despesa quando ela é executada no PO RPPS.</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85">
-        <v>869</v>
+        <v>802</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Outros Recursos Extraorçamentários</t>
+          <t>RECURSOS VINCULADOS AO RPPS - TAXA DE ADMINISTRAÇÃO</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Controle dos demais recursos financeiros extraorçamentários, como, por exemplo, retenções e consignações.</t>
+          <t>Controle dos recursos destinados ao custeio das despesas necessárias à organização e ao funcionamento da unidade gestora do RPPS, observando-se o disposto na Portaria MPS nº 402/2008 e na Portaria MF nº 464/2018, ambas alteradas pela Portaria ME nº 19.451/2020.</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86">
-        <v>880</v>
+        <v>803</v>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Recursos Próprios dos Consórcios</t>
+          <t>RECURSOS VINCULADOS AO SISTEMA DE PROTEÇÃO SOCIAL DOS MILITARES (SPSM)</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Controle dos recursos próprios dos Consórcios Públicos (utilizada pelos consórcios públicos)</t>
+          <t>Controle dos recursos vinculados ao Sistema de Proteção Social dos Militares (SPSM), com base na Lei nº 6.880/1980 (Estatuto dos Militares), alterada pela Lei nº 13.954/2019.</t>
         </is>
       </c>
     </row>
     <row r="87">
       <c r="A87">
-        <v>898</v>
+        <v>804</v>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Recursos a Classificar</t>
+          <t>DEMAIS RECURSOS PREVIDENCIÁRIOS</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Classificação temporária enquanto não se identifica a correta vinculação.</t>
+          <t>Controle de demais recursos vinculados a benefícios previdenciários, como os benefícios  mantidos sob responsabilidade financeira direta do Tesouro do ente Federativo, concedidos  em atendimento a legislações específicas e que não foram incorporados ao RPPS.</t>
         </is>
       </c>
     </row>
     <row r="88">
       <c r="A88">
+        <v>860</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>RECURSOS EXTRAORÇAMENTÁRIOS VINCULADOS A PRECATÓRIOS</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>Controle dos recursos financeiros junto aos tribunais de justiça vinculados ao pagamento de precatórios.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89">
+        <v>861</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>RECURSOS EXTRAORÇAMENTÁRIOS VINCULADOS A DEPÓSITOS JUDICIAIS</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Controle dos recursos financeiros junto aos tribunais de justiça vinculados aos depósitos judiciais.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90">
+        <v>862</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>RECURSOS DE DEPÓSITOS DE TERCEIROS</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Controle dos recursos financeiros decorrentes de depósitos de terceiros.</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91">
+        <v>869</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>OUTROS RECURSOS EXTRAORÇAMENTÁRIOS</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Controle dos demais recursos financeiros extraorçamentários, como, por exemplo, retenções e consignações.</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92">
+        <v>880</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>RECURSOS PRÓPRIOS DOS CONSÓRCIOS</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Controle dos recursos próprios dos Consórcios Públicos (utilizada pelos consórcios públicos)</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93">
+        <v>898</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>RECURSOS A CLASSIFICAR</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Classificação temporária enquanto não se identifica a correta vinculação.</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94">
         <v>899</v>
       </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>Outros Recursos Vinculados</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>OUTROS RECURSOS VINCULADOS</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
         <is>
           <t>Controle dos recursos cuja aplicação seja vinculada e não tenha sido enquadrado em outras especificações.</t>
         </is>

</xml_diff>